<commit_message>
Apresenta Compras e Cotações com dados fictícios
</commit_message>
<xml_diff>
--- a/examples/fornecedores-demo.xlsx
+++ b/examples/fornecedores-demo.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" r:id="Re59e7bec198c4c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fornecedores" sheetId="2" r:id="R0afa51704bc54f4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" r:id="Rb7cb4e1191a14051"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fornecedores" sheetId="2" r:id="Rd52c5c53c9b64163"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -604,7 +604,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Dados inteiramente fictícios para abrir, testar e apresentar o ComprasVesper sem rede corporativa.</x:v>
+        <x:v>Dados inteiramente fictícios para demonstrar o fluxo de cotações sem acesso à rede da empresa.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -900,7 +900,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f2e3a0b9cef45d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44cdab0cff774a72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Mostra Compras e Cotações com dados fictícios
Atualiza a apresentação pública, as capturas e a documentação do aplicativo.
</commit_message>
<xml_diff>
--- a/examples/fornecedores-demo.xlsx
+++ b/examples/fornecedores-demo.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" r:id="Re59e7bec198c4c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fornecedores" sheetId="2" r:id="R0afa51704bc54f4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" r:id="Rb7cb4e1191a14051"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fornecedores" sheetId="2" r:id="Rd52c5c53c9b64163"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -604,7 +604,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Dados inteiramente fictícios para abrir, testar e apresentar o ComprasVesper sem rede corporativa.</x:v>
+        <x:v>Dados inteiramente fictícios para demonstrar o fluxo de cotações sem acesso à rede da empresa.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -900,7 +900,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f2e3a0b9cef45d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44cdab0cff774a72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>